<commit_message>
added country to participants
</commit_message>
<xml_diff>
--- a/EventManager.WebUI/wwwroot/ExcelTemplates/Attendee_Template.xlsx
+++ b/EventManager.WebUI/wwwroot/ExcelTemplates/Attendee_Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashut\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashut\source\repos\EventManagerApp\EventManager.WebUI\wwwroot\ExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7941C86C-776F-4F6A-8BA7-B12BFE47AF2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79438028-E96B-4F44-9645-FEE63B0900FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{76AC1DD3-8160-4D39-BED1-F34F6A21F8EC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{76AC1DD3-8160-4D39-BED1-F34F6A21F8EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>First Name</t>
   </si>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t>Notes</t>
+  </si>
+  <si>
+    <t>Country</t>
   </si>
 </sst>
 </file>
@@ -124,10 +127,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -447,18 +446,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{051F06F1-24DD-4E31-B9AA-792A4B8F14CC}">
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.5546875" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" customWidth="1"/>
-    <col min="3" max="3" width="10.21875" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" customWidth="1"/>
-    <col min="6" max="6" width="12.21875" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="8" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -478,6 +478,9 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>